<commit_message>
Selectable company letterhead, supervisor step, per-job problems
- Ask which company (Aceken, Chemmettle, Metryscape) heads the report;
  the template no longer carries a fixed logo and the chosen company's
  logo is placed top-right of the form
- Ask the supervisor separately from the report writer
- After a job's photos, "➡️ งานนี้เสร็จ" asks whether there were
  problems/obstacles; the answer fills the form's problem column and
  shows in the summary card

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BQ8PfLcYywkQMrdgyypari
</commit_message>
<xml_diff>
--- a/line-daily-report/tools/template.xlsx
+++ b/line-daily-report/tools/template.xlsx
@@ -1168,36 +1168,6 @@
     </indexedColors>
   </colors>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
-  <oneCellAnchor>
-    <from>
-      <col>5</col>
-      <colOff>0</colOff>
-      <row>0</row>
-      <rowOff>0</rowOff>
-    </from>
-    <ext cx="1428750" cy="400050"/>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="1" name="Image 1" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
-        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </oneCellAnchor>
-</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2423,6 +2393,5 @@
   <printOptions horizontalCentered="1"/>
   <pageMargins left="0.25" right="0.25" top="0.3" bottom="0.3" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" paperSize="9" fitToHeight="1" fitToWidth="1"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Form tweaks: logo spacing, % header wrap, plan machinery order
- Taller logo row; the logo sits at the top with a gap above the form
- "เปอร์เซนต์ความคืบหน้า" breaks into two lines and its column is a bit
  wider (taken from the problem column) so the word is not cut
- In the work plan, "อื่นๆ โปรดระบุ" follows รถยนต์ directly, leaving
  the blank row at the bottom

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BQ8PfLcYywkQMrdgyypari
</commit_message>
<xml_diff>
--- a/line-daily-report/tools/template.xlsx
+++ b/line-daily-report/tools/template.xlsx
@@ -816,7 +816,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="113">
+  <cellXfs count="112">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1060,10 +1060,7 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="47" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="48" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="49" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="14" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="50" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1466,12 +1463,12 @@
     <col width="16.109375" customWidth="1" min="2" max="2"/>
     <col width="21.88671875" customWidth="1" min="3" max="3"/>
     <col width="29.109375" customWidth="1" min="4" max="4"/>
-    <col width="12.77734375" customWidth="1" min="5" max="5"/>
-    <col width="26.6640625" customWidth="1" min="6" max="6"/>
+    <col width="14.57734375" customWidth="1" min="5" max="5"/>
+    <col width="24.8640625" customWidth="1" min="6" max="6"/>
     <col width="5.44140625" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1" ht="44" customHeight="1">
+    <row r="1" ht="58" customHeight="1">
       <c r="A1" s="1" t="n"/>
       <c r="B1" s="1" t="n"/>
       <c r="C1" s="1" t="n"/>
@@ -1963,7 +1960,8 @@
       <c r="D39" s="59" t="n"/>
       <c r="E39" s="70" t="inlineStr">
         <is>
-          <t>เปอร์เซนต์ความคืบหน้า</t>
+          <t>เปอร์เซนต์
+ความคืบหน้า</t>
         </is>
       </c>
       <c r="F39" s="71" t="inlineStr">
@@ -2211,60 +2209,60 @@
     <row r="59" ht="16.8" customHeight="1">
       <c r="A59" s="97" t="n"/>
       <c r="C59" s="6" t="n"/>
-      <c r="D59" s="100" t="n"/>
+      <c r="D59" s="100" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   ☐   อื่นๆ โปรดระบุ</t>
+        </is>
+      </c>
       <c r="E59" s="95" t="n"/>
-      <c r="F59" s="101" t="n"/>
-      <c r="G59" s="102" t="n"/>
+      <c r="F59" s="101" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G59" s="18" t="n"/>
     </row>
     <row r="60" ht="16.8" customHeight="1">
-      <c r="A60" s="103" t="n"/>
+      <c r="A60" s="102" t="n"/>
       <c r="B60" s="28" t="n"/>
       <c r="C60" s="29" t="n"/>
-      <c r="D60" s="104" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   ☐   อื่นๆ โปรดระบุ</t>
-        </is>
-      </c>
+      <c r="D60" s="103" t="n"/>
       <c r="E60" s="25" t="n"/>
-      <c r="F60" s="105" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
+      <c r="F60" s="104" t="n"/>
       <c r="G60" s="25" t="n"/>
     </row>
     <row r="61" ht="16.8" customHeight="1">
-      <c r="A61" s="106" t="n"/>
-      <c r="B61" s="106" t="n"/>
-      <c r="C61" s="106" t="n"/>
-      <c r="D61" s="106" t="n"/>
-      <c r="E61" s="106" t="n"/>
-      <c r="F61" s="107" t="n"/>
-      <c r="G61" s="107" t="n"/>
+      <c r="A61" s="105" t="n"/>
+      <c r="B61" s="105" t="n"/>
+      <c r="C61" s="105" t="n"/>
+      <c r="D61" s="105" t="n"/>
+      <c r="E61" s="105" t="n"/>
+      <c r="F61" s="106" t="n"/>
+      <c r="G61" s="106" t="n"/>
     </row>
     <row r="62" ht="16.8" customHeight="1">
-      <c r="A62" s="106" t="n"/>
-      <c r="B62" s="106" t="n"/>
-      <c r="C62" s="106" t="n"/>
-      <c r="D62" s="106" t="n"/>
-      <c r="E62" s="106" t="n"/>
-      <c r="F62" s="107" t="n"/>
-      <c r="G62" s="107" t="n"/>
+      <c r="A62" s="105" t="n"/>
+      <c r="B62" s="105" t="n"/>
+      <c r="C62" s="105" t="n"/>
+      <c r="D62" s="105" t="n"/>
+      <c r="E62" s="105" t="n"/>
+      <c r="F62" s="106" t="n"/>
+      <c r="G62" s="106" t="n"/>
     </row>
     <row r="63" ht="30.6" customHeight="1">
-      <c r="A63" s="108" t="inlineStr">
+      <c r="A63" s="107" t="inlineStr">
         <is>
           <t>ลงชื่อผู้บันทึก</t>
         </is>
       </c>
-      <c r="B63" s="109" t="n"/>
-      <c r="C63" s="108" t="inlineStr">
+      <c r="B63" s="108" t="n"/>
+      <c r="C63" s="107" t="inlineStr">
         <is>
           <t>ลงชื่อผู้ควบคุมงาน</t>
         </is>
       </c>
-      <c r="D63" s="109" t="n"/>
-      <c r="E63" s="108" t="inlineStr">
+      <c r="D63" s="108" t="n"/>
+      <c r="E63" s="107" t="inlineStr">
         <is>
           <t>ลงชื่อลูกค้า:</t>
         </is>
@@ -2273,28 +2271,28 @@
       <c r="G63" s="65" t="n"/>
     </row>
     <row r="64" ht="20.4" customHeight="1">
-      <c r="A64" s="108" t="inlineStr">
+      <c r="A64" s="107" t="inlineStr">
         <is>
           <t>วันที่/Date:</t>
         </is>
       </c>
-      <c r="B64" s="110" t="n"/>
-      <c r="C64" s="108" t="inlineStr">
+      <c r="B64" s="109" t="n"/>
+      <c r="C64" s="107" t="inlineStr">
         <is>
           <t>วันที่/Date:</t>
         </is>
       </c>
-      <c r="D64" s="111" t="n"/>
-      <c r="E64" s="108" t="inlineStr">
+      <c r="D64" s="110" t="n"/>
+      <c r="E64" s="107" t="inlineStr">
         <is>
           <t>วันที่/Date:</t>
         </is>
       </c>
-      <c r="F64" s="110" t="n"/>
+      <c r="F64" s="109" t="n"/>
       <c r="G64" s="73" t="n"/>
     </row>
     <row r="65" ht="20.4" customHeight="1">
-      <c r="A65" s="112" t="inlineStr">
+      <c r="A65" s="111" t="inlineStr">
         <is>
           <t>FM_Daily Report_R02</t>
         </is>
@@ -2307,7 +2305,7 @@
       <c r="G65" s="1" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="81">
+  <mergeCells count="82">
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="D8:G8"/>
     <mergeCell ref="A57:C57"/>
@@ -2372,6 +2370,7 @@
     <mergeCell ref="A56:C56"/>
     <mergeCell ref="A43:D43"/>
     <mergeCell ref="F40:G40"/>
+    <mergeCell ref="F59:G59"/>
     <mergeCell ref="A40:D40"/>
     <mergeCell ref="F55:G55"/>
     <mergeCell ref="F12:G12"/>

</xml_diff>